<commit_message>
Added bunch of things
</commit_message>
<xml_diff>
--- a/simulation_results.xlsx
+++ b/simulation_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Total Steps</t>
+          <t>Total Steps (All Attempts)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>352</v>
+        <v>237</v>
       </c>
       <c r="F2" t="n">
-        <v>961</v>
+        <v>756</v>
       </c>
       <c r="G2" t="n">
-        <v>2.566139999544248</v>
+        <v>1.97379200017167</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -515,13 +515,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>350</v>
+        <v>233</v>
       </c>
       <c r="F3" t="n">
-        <v>5491</v>
+        <v>3552</v>
       </c>
       <c r="G3" t="n">
-        <v>8.861956999680842</v>
+        <v>5.534724999051832</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -543,16 +543,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="F4" t="n">
-        <v>2051</v>
+        <v>2037</v>
       </c>
       <c r="G4" t="n">
-        <v>5.026944999372063</v>
+        <v>4.574722002871567</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -571,16 +571,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>40</v>
+        <v>296</v>
       </c>
       <c r="F5" t="n">
-        <v>53248</v>
+        <v>3679</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9208800001943018</v>
+        <v>5.634200998429151</v>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -599,16 +599,16 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>292</v>
       </c>
       <c r="F6" t="n">
-        <v>12060</v>
+        <v>7561</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>17.86767700377823</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -627,16 +627,16 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>329</v>
+        <v>249</v>
       </c>
       <c r="F7" t="n">
-        <v>10212</v>
+        <v>9762</v>
       </c>
       <c r="G7" t="n">
-        <v>15.68751900003917</v>
+        <v>14.23200899989752</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -655,13 +655,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F8" t="n">
-        <v>643</v>
+        <v>1158</v>
       </c>
       <c r="G8" t="n">
-        <v>1.72281899904192</v>
+        <v>2.569874999608146</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -683,13 +683,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F9" t="n">
-        <v>3530</v>
+        <v>3879</v>
       </c>
       <c r="G9" t="n">
-        <v>5.269269000564236</v>
+        <v>5.473499999425258</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>102</v>
+        <v>187</v>
       </c>
       <c r="F10" t="n">
-        <v>29930</v>
+        <v>538</v>
       </c>
       <c r="G10" t="n">
-        <v>0.6753079996997258</v>
+        <v>1.305898000282468</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
@@ -739,16 +739,16 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>108</v>
+        <v>238</v>
       </c>
       <c r="F11" t="n">
-        <v>18519</v>
+        <v>3940</v>
       </c>
       <c r="G11" t="n">
-        <v>2.099670001371123</v>
+        <v>5.892465001124947</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>154</v>
+        <v>261</v>
       </c>
       <c r="F12" t="n">
-        <v>6760</v>
+        <v>2032</v>
       </c>
       <c r="G12" t="n">
-        <v>1.877531000445742</v>
+        <v>4.523215001427161</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
@@ -795,13 +795,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>415</v>
       </c>
       <c r="F13" t="n">
-        <v>11520</v>
+        <v>50916</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>72.60417599263747</v>
       </c>
       <c r="H13" t="n">
         <v>3</v>
@@ -823,13 +823,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>251</v>
+        <v>291</v>
       </c>
       <c r="F14" t="n">
-        <v>712</v>
+        <v>1324</v>
       </c>
       <c r="G14" t="n">
-        <v>1.580517999627773</v>
+        <v>2.793490000840393</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -851,13 +851,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>233</v>
+        <v>291</v>
       </c>
       <c r="F15" t="n">
-        <v>3309</v>
+        <v>3956</v>
       </c>
       <c r="G15" t="n">
-        <v>4.501902000356495</v>
+        <v>5.601148999630823</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -879,16 +879,16 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>351</v>
+        <v>295</v>
       </c>
       <c r="F16" t="n">
-        <v>1538</v>
+        <v>5123</v>
       </c>
       <c r="G16" t="n">
-        <v>3.154230999825813</v>
+        <v>11.04262299850234</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -907,16 +907,16 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>98</v>
+        <v>324</v>
       </c>
       <c r="F17" t="n">
-        <v>42586</v>
+        <v>3761</v>
       </c>
       <c r="G17" t="n">
-        <v>1.942753000093944</v>
+        <v>5.743090999203559</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -935,16 +935,16 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>311</v>
       </c>
       <c r="F18" t="n">
-        <v>35012</v>
+        <v>54299</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>115.27938800009</v>
       </c>
       <c r="H18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -963,13 +963,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>90</v>
+        <v>255</v>
       </c>
       <c r="F19" t="n">
-        <v>11477</v>
+        <v>19862</v>
       </c>
       <c r="G19" t="n">
-        <v>9.078701999897021</v>
+        <v>28.89261199834436</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
@@ -991,13 +991,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>269</v>
+        <v>250</v>
       </c>
       <c r="F20" t="n">
-        <v>1095</v>
+        <v>594</v>
       </c>
       <c r="G20" t="n">
-        <v>2.311836999069783</v>
+        <v>1.344710000012128</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1019,13 +1019,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>267</v>
+        <v>250</v>
       </c>
       <c r="F21" t="n">
-        <v>3852</v>
+        <v>3320</v>
       </c>
       <c r="G21" t="n">
-        <v>5.301238999891211</v>
+        <v>4.656315999454819</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1047,16 +1047,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>95</v>
+        <v>267</v>
       </c>
       <c r="F22" t="n">
-        <v>15699</v>
+        <v>1259</v>
       </c>
       <c r="G22" t="n">
-        <v>0.7371040001089568</v>
+        <v>2.866819001610565</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1075,16 +1075,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>146</v>
+        <v>263</v>
       </c>
       <c r="F23" t="n">
-        <v>6251</v>
+        <v>3919</v>
       </c>
       <c r="G23" t="n">
-        <v>2.975921999677666</v>
+        <v>5.528367000806611</v>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>146</v>
+        <v>400</v>
       </c>
       <c r="F24" t="n">
-        <v>2396</v>
+        <v>11368</v>
       </c>
       <c r="G24" t="n">
-        <v>1.331760999619291</v>
+        <v>24.98872800333629</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1131,16 +1131,16 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>164</v>
+        <v>206</v>
       </c>
       <c r="F25" t="n">
-        <v>13365</v>
+        <v>9716</v>
       </c>
       <c r="G25" t="n">
-        <v>12.20747200068217</v>
+        <v>14.19776400234696</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -1159,13 +1159,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F26" t="n">
-        <v>766</v>
+        <v>1033</v>
       </c>
       <c r="G26" t="n">
-        <v>1.769444999808911</v>
+        <v>2.228809998996439</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1187,13 +1187,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="F27" t="n">
-        <v>4191</v>
+        <v>4276</v>
       </c>
       <c r="G27" t="n">
-        <v>6.069088000003831</v>
+        <v>6.253429999560467</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1215,16 +1215,16 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>211</v>
+        <v>365</v>
       </c>
       <c r="F28" t="n">
-        <v>1858</v>
+        <v>35173</v>
       </c>
       <c r="G28" t="n">
-        <v>3.476507999494061</v>
+        <v>74.59018200279388</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -1243,16 +1243,16 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>309</v>
+        <v>374</v>
       </c>
       <c r="F29" t="n">
-        <v>10806</v>
+        <v>26089</v>
       </c>
       <c r="G29" t="n">
-        <v>13.26556499907383</v>
+        <v>38.53939400050876</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1271,13 +1271,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>98</v>
+        <v>244</v>
       </c>
       <c r="F30" t="n">
-        <v>11492</v>
+        <v>5460</v>
       </c>
       <c r="G30" t="n">
-        <v>0.6053829997654248</v>
+        <v>12.11295099892595</v>
       </c>
       <c r="H30" t="n">
         <v>2</v>
@@ -1299,184 +1299,16 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>194</v>
+        <v>417</v>
       </c>
       <c r="F31" t="n">
-        <v>22400</v>
+        <v>51886</v>
       </c>
       <c r="G31" t="n">
-        <v>24.61016599863797</v>
+        <v>72.58525599991117</v>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>6</v>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>260</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1136</v>
-      </c>
-      <c r="G32" t="n">
-        <v>2.606355000807525</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>6</v>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>256</v>
-      </c>
-      <c r="F33" t="n">
-        <v>3532</v>
-      </c>
-      <c r="G33" t="n">
-        <v>5.394905999764887</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>6</v>
-      </c>
-      <c r="B34" t="n">
-        <v>2</v>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>175</v>
-      </c>
-      <c r="F34" t="n">
-        <v>10784</v>
-      </c>
-      <c r="G34" t="n">
-        <v>4.475466998883348</v>
-      </c>
-      <c r="H34" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>6</v>
-      </c>
-      <c r="B35" t="n">
-        <v>2</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>318</v>
-      </c>
-      <c r="F35" t="n">
-        <v>5740</v>
-      </c>
-      <c r="G35" t="n">
-        <v>6.824044000040885</v>
-      </c>
-      <c r="H35" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>6</v>
-      </c>
-      <c r="B36" t="n">
-        <v>3</v>
-      </c>
-      <c r="C36" t="n">
-        <v>2</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>96</v>
-      </c>
-      <c r="F36" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0.4936919999636302</v>
-      </c>
-      <c r="H36" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>6</v>
-      </c>
-      <c r="B37" t="n">
-        <v>3</v>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>96</v>
-      </c>
-      <c r="F37" t="n">
-        <v>4397</v>
-      </c>
-      <c r="G37" t="n">
-        <v>1.332598000317375</v>
-      </c>
-      <c r="H37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1490,7 +1322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1546,7 +1378,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -1570,7 +1402,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4">
@@ -1594,7 +1426,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>283</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5">
@@ -1618,7 +1450,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -1642,7 +1474,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
@@ -1666,7 +1498,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>283</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8">
@@ -1686,11 +1518,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1714,7 +1546,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>95</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
@@ -1738,7 +1570,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>120</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">
@@ -1758,11 +1590,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -1782,11 +1614,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>52</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13">
@@ -1806,11 +1638,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>110</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14">
@@ -1834,7 +1666,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>142</v>
       </c>
     </row>
     <row r="15">
@@ -1858,7 +1690,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>163</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -1878,11 +1710,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>121</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17">
@@ -1906,7 +1738,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18">
@@ -1926,11 +1758,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>163</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19">
@@ -1954,7 +1786,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20">
@@ -1978,7 +1810,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21">
@@ -2002,7 +1834,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>155</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22">
@@ -2026,7 +1858,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>147</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23">
@@ -2050,7 +1882,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24">
@@ -2074,7 +1906,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>155</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25">
@@ -2098,7 +1930,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>147</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26">
@@ -2122,7 +1954,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27">
@@ -2142,11 +1974,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28">
@@ -2166,11 +1998,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>79</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29">
@@ -2194,7 +2026,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30">
@@ -2218,7 +2050,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31">
@@ -2238,11 +2070,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>318</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32">
@@ -2266,7 +2098,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33">
@@ -2290,7 +2122,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34">
@@ -2314,7 +2146,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>165</v>
+        <v>185</v>
       </c>
     </row>
     <row r="35">
@@ -2338,7 +2170,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36">
@@ -2362,7 +2194,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>46</v>
+        <v>188</v>
       </c>
     </row>
     <row r="37">
@@ -2386,7 +2218,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>154</v>
+        <v>185</v>
       </c>
     </row>
     <row r="38">
@@ -2410,7 +2242,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>71</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39">
@@ -2434,7 +2266,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>107</v>
+        <v>139</v>
       </c>
     </row>
     <row r="40">
@@ -2458,7 +2290,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>154</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41">
@@ -2482,7 +2314,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>71</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42">
@@ -2506,7 +2338,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>107</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43">
@@ -2530,7 +2362,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>154</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44">
@@ -2554,7 +2386,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45">
@@ -2578,7 +2410,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="46">
@@ -2598,11 +2430,11 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>280</v>
+        <v>160</v>
       </c>
     </row>
     <row r="47">
@@ -2626,7 +2458,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48">
@@ -2650,7 +2482,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="49">
@@ -2670,11 +2502,11 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>199</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50">
@@ -2698,7 +2530,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
@@ -2718,11 +2550,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>75</v>
+        <v>153</v>
       </c>
     </row>
     <row r="52">
@@ -2746,7 +2578,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>149</v>
+        <v>182</v>
       </c>
     </row>
     <row r="53">
@@ -2770,7 +2602,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54">
@@ -2794,7 +2626,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>97</v>
+        <v>153</v>
       </c>
     </row>
     <row r="55">
@@ -2818,7 +2650,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>86</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56">
@@ -2842,7 +2674,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="57">
@@ -2866,7 +2698,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58">
@@ -2890,7 +2722,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>153</v>
+        <v>188</v>
       </c>
     </row>
     <row r="59">
@@ -2914,7 +2746,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="60">
@@ -2938,7 +2770,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="61">
@@ -2962,7 +2794,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>153</v>
+        <v>188</v>
       </c>
     </row>
     <row r="62">
@@ -2982,11 +2814,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
     </row>
     <row r="63">
@@ -3010,7 +2842,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
     </row>
     <row r="64">
@@ -3030,11 +2862,11 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>185</v>
+        <v>168</v>
       </c>
     </row>
     <row r="65">
@@ -3058,7 +2890,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>86</v>
+        <v>31</v>
       </c>
     </row>
     <row r="66">
@@ -3082,7 +2914,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67">
@@ -3102,11 +2934,11 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>324</v>
+        <v>168</v>
       </c>
     </row>
     <row r="68">
@@ -3130,7 +2962,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="69">
@@ -3154,7 +2986,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>81</v>
+        <v>137</v>
       </c>
     </row>
     <row r="70">
@@ -3174,11 +3006,11 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>184</v>
+        <v>223</v>
       </c>
     </row>
     <row r="71">
@@ -3202,7 +3034,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="72">
@@ -3226,7 +3058,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>56</v>
+        <v>98</v>
       </c>
     </row>
     <row r="73">
@@ -3246,11 +3078,11 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>184</v>
+        <v>68</v>
       </c>
     </row>
     <row r="74">
@@ -3274,7 +3106,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="75">
@@ -3298,7 +3130,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>102</v>
+        <v>139</v>
       </c>
     </row>
     <row r="76">
@@ -3322,7 +3154,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>187</v>
+        <v>238</v>
       </c>
     </row>
     <row r="77">
@@ -3346,7 +3178,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="78">
@@ -3370,7 +3202,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>102</v>
+        <v>139</v>
       </c>
     </row>
     <row r="79">
@@ -3394,7 +3226,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>187</v>
+        <v>238</v>
       </c>
     </row>
     <row r="80">
@@ -3418,7 +3250,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>29</v>
+        <v>83</v>
       </c>
     </row>
     <row r="81">
@@ -3438,11 +3270,11 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="82">
@@ -3462,11 +3294,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>268</v>
+        <v>191</v>
       </c>
     </row>
     <row r="83">
@@ -3486,11 +3318,11 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="84">
@@ -3510,11 +3342,11 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="85">
@@ -3534,11 +3366,11 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>268</v>
+        <v>204</v>
       </c>
     </row>
     <row r="86">
@@ -3558,11 +3390,11 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>DIED</t>
+          <t>FINISHED</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>109</v>
+        <v>50</v>
       </c>
     </row>
     <row r="87">
@@ -3586,7 +3418,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>126</v>
+        <v>157</v>
       </c>
     </row>
     <row r="88">
@@ -3606,11 +3438,11 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>104</v>
+        <v>40</v>
       </c>
     </row>
     <row r="89">
@@ -3634,7 +3466,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="90">
@@ -3654,11 +3486,11 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>DIED</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>264</v>
+        <v>155</v>
       </c>
     </row>
     <row r="91">
@@ -3682,439 +3514,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>6</v>
-      </c>
-      <c r="B92" t="n">
-        <v>1</v>
-      </c>
-      <c r="C92" t="n">
-        <v>1</v>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F92" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>6</v>
-      </c>
-      <c r="B93" t="n">
-        <v>1</v>
-      </c>
-      <c r="C93" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F93" t="n">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>6</v>
-      </c>
-      <c r="B94" t="n">
-        <v>1</v>
-      </c>
-      <c r="C94" t="n">
-        <v>3</v>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F94" t="n">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>6</v>
-      </c>
-      <c r="B95" t="n">
-        <v>1</v>
-      </c>
-      <c r="C95" t="n">
-        <v>1</v>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F95" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>6</v>
-      </c>
-      <c r="B96" t="n">
-        <v>1</v>
-      </c>
-      <c r="C96" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F96" t="n">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>6</v>
-      </c>
-      <c r="B97" t="n">
-        <v>1</v>
-      </c>
-      <c r="C97" t="n">
-        <v>3</v>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F97" t="n">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>6</v>
-      </c>
-      <c r="B98" t="n">
-        <v>2</v>
-      </c>
-      <c r="C98" t="n">
-        <v>1</v>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F98" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>6</v>
-      </c>
-      <c r="B99" t="n">
-        <v>2</v>
-      </c>
-      <c r="C99" t="n">
-        <v>2</v>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F99" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>6</v>
-      </c>
-      <c r="B100" t="n">
-        <v>2</v>
-      </c>
-      <c r="C100" t="n">
-        <v>3</v>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>DIED</t>
-        </is>
-      </c>
-      <c r="F100" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>6</v>
-      </c>
-      <c r="B101" t="n">
-        <v>2</v>
-      </c>
-      <c r="C101" t="n">
-        <v>1</v>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>DIED</t>
-        </is>
-      </c>
-      <c r="F101" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>6</v>
-      </c>
-      <c r="B102" t="n">
-        <v>2</v>
-      </c>
-      <c r="C102" t="n">
-        <v>2</v>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F102" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>6</v>
-      </c>
-      <c r="B103" t="n">
-        <v>2</v>
-      </c>
-      <c r="C103" t="n">
-        <v>3</v>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F103" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>6</v>
-      </c>
-      <c r="B104" t="n">
-        <v>3</v>
-      </c>
-      <c r="C104" t="n">
-        <v>1</v>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>DIED</t>
-        </is>
-      </c>
-      <c r="F104" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>6</v>
-      </c>
-      <c r="B105" t="n">
-        <v>3</v>
-      </c>
-      <c r="C105" t="n">
-        <v>2</v>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>DIED</t>
-        </is>
-      </c>
-      <c r="F105" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>6</v>
-      </c>
-      <c r="B106" t="n">
-        <v>3</v>
-      </c>
-      <c r="C106" t="n">
-        <v>3</v>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>AStar</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F106" t="n">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>6</v>
-      </c>
-      <c r="B107" t="n">
-        <v>3</v>
-      </c>
-      <c r="C107" t="n">
-        <v>1</v>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>DIED</t>
-        </is>
-      </c>
-      <c r="F107" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>6</v>
-      </c>
-      <c r="B108" t="n">
-        <v>3</v>
-      </c>
-      <c r="C108" t="n">
-        <v>2</v>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>DIED</t>
-        </is>
-      </c>
-      <c r="F108" t="n">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>6</v>
-      </c>
-      <c r="B109" t="n">
-        <v>3</v>
-      </c>
-      <c r="C109" t="n">
-        <v>3</v>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>BFS</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="F109" t="n">
-        <v>104</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>